<commit_message>
Mentor roster: preload staging, expanded panel, and admin UI copy
- Rework expanded mentor row: contact first, program/staging editors, notes last; staging vs live contact layout.

- Mentor preload import/registry plumbing, migration 122, template and lib helpers.

- Button and section labels: Title Case and clarified helper text.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/public/frontier-mentor-roster-import-template.xlsx
+++ b/public/frontier-mentor-roster-import-template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\svenf\crewrules\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{29B1F2F6-046F-4B9A-8A4F-E07CD7D1DC65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{3453FA67-A8C2-4C5E-937E-F64F02BD93AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-57720" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BEE25EB5-B863-415F-AAF3-BD0349D0BAE6}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{BEE25EB5-B863-415F-AAF3-BD0349D0BAE6}"/>
   </bookViews>
   <sheets>
     <sheet name="mentoring-mentee-import-Try2" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="5" uniqueCount="5">
+<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="7" uniqueCount="7">
   <si>
     <t>mentor_employee_number</t>
   </si>
@@ -39,14 +39,20 @@
     <t>mentor_phone_number</t>
   </si>
   <si>
-    <t>mentor_email_@flyfrontier.com</t>
+    <t>mentor_email_@for.mentoring</t>
+  </si>
+  <si>
+    <t>role</t>
+  </si>
+  <si>
+    <t>crew_base</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -181,6 +187,17 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="34">
     <fill>
@@ -369,7 +386,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="13">
     <border>
       <start/>
       <end/>
@@ -481,6 +498,49 @@
       </top>
       <bottom style="double">
         <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <start style="thin">
+        <color rgb="FF000000"/>
+      </start>
+      <end style="thin">
+        <color rgb="FF000000"/>
+      </end>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <start style="thin">
+        <color rgb="FF000000"/>
+      </start>
+      <end/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <start style="thin">
+        <color indexed="64"/>
+      </start>
+      <end style="thin">
+        <color indexed="64"/>
+      </end>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -529,10 +589,30 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="14" fontId="0" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -908,31 +988,48 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19CE3EA6-B8E4-4529-86C0-6157932FF605}">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="22.54296875" customWidth="1"/>
-    <col min="2" max="2" width="23.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="27.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.54296875" style="6" customWidth="1"/>
+    <col min="2" max="2" width="23.54296875" style="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.81640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="27.81640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="32.81640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="8.7265625" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="8" t="s">
         <v>1</v>
       </c>
+      <c r="F1" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat(mentoring): mentor categories, preload import, roster & import docs
- Add mentor_registry.mentor.categories migration (123)

- Preload CSV: program/status/seat columns; seat precedes role for position

- Import: upsert mentor_registry from program/status when preload unmatched

- Roster: categories in program pill; wire mentor_categories for profile rows

- Mentor import page: grouped helper copy, example row, template xlsx

- Includes other modified files in workspace (waitlist, admin page, etc.)

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/public/frontier-mentor-roster-import-template.xlsx
+++ b/public/frontier-mentor-roster-import-template.xlsx
@@ -8,24 +8,35 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\svenf\crewrules\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{3453FA67-A8C2-4C5E-937E-F64F02BD93AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5970238D-109D-49F6-A33B-71EF184AD125}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{BEE25EB5-B863-415F-AAF3-BD0349D0BAE6}"/>
   </bookViews>
   <sheets>
     <sheet name="mentoring-mentee-import-Try2" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
       <x14:workbookPr/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="7" uniqueCount="7">
+<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="11" uniqueCount="11">
   <si>
     <t>mentor_employee_number</t>
   </si>
@@ -42,17 +53,29 @@
     <t>mentor_email_@for.mentoring</t>
   </si>
   <si>
-    <t>role</t>
+    <t>crew_base</t>
   </si>
   <si>
-    <t>crew_base</t>
+    <t>mentor_email_@flyfrontier.com</t>
+  </si>
+  <si>
+    <t>Scott Peters</t>
+  </si>
+  <si>
+    <t>Seat</t>
+  </si>
+  <si>
+    <t>program</t>
+  </si>
+  <si>
+    <t>status</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -198,6 +221,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="34">
     <fill>
@@ -386,7 +415,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="10">
     <border>
       <start/>
       <end/>
@@ -501,49 +530,6 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <start style="thin">
-        <color rgb="FF000000"/>
-      </start>
-      <end style="thin">
-        <color rgb="FF000000"/>
-      </end>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <start style="thin">
-        <color rgb="FF000000"/>
-      </start>
-      <end/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <start style="thin">
-        <color indexed="64"/>
-      </start>
-      <end style="thin">
-        <color indexed="64"/>
-      </end>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -589,28 +575,27 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -988,48 +973,65 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19CE3EA6-B8E4-4529-86C0-6157932FF605}">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="22.54296875" style="6" customWidth="1"/>
-    <col min="2" max="2" width="23.54296875" style="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.81640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="27.81640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="32.81640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="8.7265625" style="6"/>
+    <col min="1" max="1" width="22.54296875" style="9" customWidth="1"/>
+    <col min="2" max="2" width="23.54296875" style="9" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.81640625" style="9" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.81640625" style="9" customWidth="1"/>
+    <col min="5" max="5" width="27.81640625" style="9" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="32.81640625" style="9" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="11.1796875" style="9" customWidth="1"/>
+    <col min="9" max="10" width="8.7265625" style="9"/>
+    <col min="11" max="16384" width="8.7265625" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="F1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="G1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="8" t="s">
-        <v>6</v>
+    </row>
+    <row r="2" spans="1:10" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.4">
+      <c r="A2" s="5" t="s">
+        <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="2"/>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="7"/>
+      <c r="I2" s="5"/>
+      <c r="J2" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>